<commit_message>
updates for 95% fisherian intervals
I finished the fisherian intervals for all the important primary and secondary genes
</commit_message>
<xml_diff>
--- a/primary genes/lung_genes_primary_results.xlsx
+++ b/primary genes/lung_genes_primary_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anqiwang/Documents/GitHub/Ozone-and-Lung-Functions/primary genes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C27727-ACDB-D644-8B0B-5B6009C2BB19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419288F2-B0F7-6A49-AD74-C6E42F519EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3440" yWindow="700" windowWidth="20740" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13080" yWindow="0" windowWidth="15720" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>